<commit_message>
Revamp ecosystem solutions, update EN pages, add new assets
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/prop/translation/solutions.xlsx.xlsx
+++ b/prop/translation/solutions.xlsx.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20752" windowHeight="10080" activeTab="1"/>
+    <workbookView windowWidth="20752" windowHeight="10080"/>
   </bookViews>
   <sheets>
     <sheet name="Industry Solutions (行业应用方案)" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,13 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="95">
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Inter"/>
+        <charset val="134"/>
+      </rPr>
       <t>English Name (</t>
     </r>
     <r>
@@ -56,6 +63,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Inter"/>
+        <charset val="134"/>
+      </rPr>
       <t>Chinese Name (</t>
     </r>
     <r>
@@ -369,7 +383,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -388,13 +402,6 @@
       <sz val="11"/>
       <name val="Inter"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -878,156 +885,153 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1400,205 +1404,205 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1625,164 +1629,164 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>94</v>
       </c>
     </row>

</xml_diff>